<commit_message>
Added new RDF data schemes and visual schemes for environment-table43-44, and fixed XLSX spreadsheets for environment-table43-44
</commit_message>
<xml_diff>
--- a/sources/table_normalization/xlsx/environment-table43.xlsx
+++ b/sources/table_normalization/xlsx/environment-table43.xlsx
@@ -237,7 +237,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -255,7 +255,6 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -933,9 +932,9 @@
       <c r="A12" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="6"/>
-      <c r="C12" s="6"/>
-      <c r="D12" s="6"/>
+      <c r="B12" s="2"/>
+      <c r="C12" s="2"/>
+      <c r="D12" s="2"/>
       <c r="E12" s="5">
         <f>AVERAGE(E2:E11)</f>
         <v>0.11600000000000001</v>
@@ -946,9 +945,9 @@
       <c r="A13" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="B13" s="6"/>
-      <c r="C13" s="6"/>
-      <c r="D13" s="6"/>
+      <c r="B13" s="2"/>
+      <c r="C13" s="2"/>
+      <c r="D13" s="2"/>
       <c r="E13" s="5">
         <f>STDEV(E2:E11)</f>
         <v>1.09134168190657</v>
@@ -959,9 +958,9 @@
       <c r="A14" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="B14" s="6"/>
-      <c r="C14" s="6"/>
-      <c r="D14" s="6"/>
+      <c r="B14" s="2"/>
+      <c r="C14" s="2"/>
+      <c r="D14" s="2"/>
       <c r="E14" s="5">
         <f>E13/SQRT(10)</f>
         <v>0.345112542030374</v>
@@ -1148,9 +1147,9 @@
       <c r="A26" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="B26" s="6"/>
-      <c r="C26" s="6"/>
-      <c r="D26" s="6"/>
+      <c r="B26" s="2"/>
+      <c r="C26" s="2"/>
+      <c r="D26" s="2"/>
       <c r="E26" s="5">
         <f>AVERAGE(E16:E25)</f>
         <v>2.2919999999999998</v>
@@ -1160,9 +1159,9 @@
       <c r="A27" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="B27" s="6"/>
-      <c r="C27" s="6"/>
-      <c r="D27" s="6"/>
+      <c r="B27" s="2"/>
+      <c r="C27" s="2"/>
+      <c r="D27" s="2"/>
       <c r="E27" s="5">
         <f>STDEV(E16:E25)</f>
         <v>1.03954904753081</v>
@@ -1172,9 +1171,9 @@
       <c r="A28" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="B28" s="6"/>
-      <c r="C28" s="6"/>
-      <c r="D28" s="6"/>
+      <c r="B28" s="2"/>
+      <c r="C28" s="2"/>
+      <c r="D28" s="2"/>
       <c r="E28" s="5">
         <f>E27/SQRT(10)</f>
         <v>0.32873427296560098</v>
@@ -1462,9 +1461,9 @@
       <c r="A46" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="B46" s="6"/>
-      <c r="C46" s="6"/>
-      <c r="D46" s="6"/>
+      <c r="B46" s="2"/>
+      <c r="C46" s="2"/>
+      <c r="D46" s="2"/>
       <c r="E46" s="5">
         <f>AVERAGE(E30:E45)</f>
         <v>4.8187499999999996</v>
@@ -1474,9 +1473,9 @@
       <c r="A47" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="B47" s="6"/>
-      <c r="C47" s="6"/>
-      <c r="D47" s="6"/>
+      <c r="B47" s="2"/>
+      <c r="C47" s="2"/>
+      <c r="D47" s="2"/>
       <c r="E47" s="5">
         <f>STDEV(E30:E45)</f>
         <v>1.15848104573762</v>
@@ -1486,9 +1485,9 @@
       <c r="A48" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="B48" s="6"/>
-      <c r="C48" s="6"/>
-      <c r="D48" s="6"/>
+      <c r="B48" s="2"/>
+      <c r="C48" s="2"/>
+      <c r="D48" s="2"/>
       <c r="E48" s="5">
         <f>E47/SQRT(16)</f>
         <v>0.289620261434405</v>
@@ -1742,9 +1741,9 @@
       <c r="A64" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="B64" s="6"/>
-      <c r="C64" s="6"/>
-      <c r="D64" s="6"/>
+      <c r="B64" s="2"/>
+      <c r="C64" s="2"/>
+      <c r="D64" s="2"/>
       <c r="E64" s="5">
         <f>AVERAGE(E50:E63)</f>
         <v>3.2149999999999999</v>
@@ -1754,9 +1753,9 @@
       <c r="A65" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="B65" s="6"/>
-      <c r="C65" s="6"/>
-      <c r="D65" s="6"/>
+      <c r="B65" s="2"/>
+      <c r="C65" s="2"/>
+      <c r="D65" s="2"/>
       <c r="E65" s="5">
         <f>STDEV(E50:E63)</f>
         <v>1.6240393610235699</v>
@@ -1766,9 +1765,9 @@
       <c r="A66" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="B66" s="6"/>
-      <c r="C66" s="6"/>
-      <c r="D66" s="6"/>
+      <c r="B66" s="2"/>
+      <c r="C66" s="2"/>
+      <c r="D66" s="2"/>
       <c r="E66" s="5">
         <f>E65/SQRT(14)</f>
         <v>0.434042776541819</v>
@@ -1920,9 +1919,9 @@
       <c r="A76" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="B76" s="6"/>
-      <c r="C76" s="6"/>
-      <c r="D76" s="6"/>
+      <c r="B76" s="2"/>
+      <c r="C76" s="2"/>
+      <c r="D76" s="2"/>
       <c r="E76" s="5">
         <f>AVERAGE(E68:E75)</f>
         <v>5.8375000000000004</v>
@@ -1932,9 +1931,9 @@
       <c r="A77" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="B77" s="6"/>
-      <c r="C77" s="6"/>
-      <c r="D77" s="6"/>
+      <c r="B77" s="2"/>
+      <c r="C77" s="2"/>
+      <c r="D77" s="2"/>
       <c r="E77" s="5">
         <f>STDEV(E68:E75)</f>
         <v>0.81048045715400896</v>
@@ -1944,9 +1943,9 @@
       <c r="A78" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="B78" s="6"/>
-      <c r="C78" s="6"/>
-      <c r="D78" s="6"/>
+      <c r="B78" s="2"/>
+      <c r="C78" s="2"/>
+      <c r="D78" s="2"/>
       <c r="E78" s="5">
         <f>E77/SQRT(8)</f>
         <v>0.28654811363638599</v>
@@ -2115,9 +2114,6 @@
       <c r="A89" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="B89" s="7"/>
-      <c r="C89" s="7"/>
-      <c r="D89" s="7"/>
       <c r="E89" s="5">
         <f>AVERAGE(E80:E88)</f>
         <v>5.3733333333333304</v>
@@ -2127,9 +2123,6 @@
       <c r="A90" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="B90" s="7"/>
-      <c r="C90" s="7"/>
-      <c r="D90" s="7"/>
       <c r="E90" s="5">
         <f>STDEV(E80:E88)</f>
         <v>1.30369666717377</v>
@@ -2139,9 +2132,6 @@
       <c r="A91" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="B91" s="7"/>
-      <c r="C91" s="7"/>
-      <c r="D91" s="7"/>
       <c r="E91" s="5">
         <f>E90/SQRT(9)</f>
         <v>0.43456555572459099</v>

</xml_diff>